<commit_message>
NDC Ajout masse détaillée masses plat et profilé
</commit_message>
<xml_diff>
--- a/VALIDATION/CAS SFS03/Cas SFS03.xlsx
+++ b/VALIDATION/CAS SFS03/Cas SFS03.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV23\VALIDATION\CAS SFS03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4EB0C6-6293-4380-9344-8BDCD9A22DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57698C3C-A508-4B39-B0FE-889B56E4073F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="21600" windowHeight="13950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="I6" s="94">
         <f>D55</f>
-        <v>10.805430827848586</v>
+        <v>10.989368327848585</v>
       </c>
       <c r="J6" t="s">
         <v>7</v>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="J13" s="9">
         <f>qG*LL^2/8</f>
-        <v>66.183263820572591</v>
+        <v>67.30988100807258</v>
       </c>
       <c r="K13" s="12" t="s">
         <v>18</v>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="J14" s="80">
         <f>qG*LL/2</f>
-        <v>37.819007897470051</v>
+        <v>38.462789147470048</v>
       </c>
       <c r="K14" s="15" t="s">
         <v>8</v>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="J23" s="48">
         <f>GammaG*MEdG+GammaQ*(MEd_Q1+Psi_0*MEd_Q2)</f>
-        <v>227.15990615777301</v>
+        <v>228.68083936089801</v>
       </c>
       <c r="K23" s="31" t="s">
         <v>18</v>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="J24" s="48">
         <f>GammaG*VEdG+GammaQ*(VEd_Q1+Psi_0*VEd_Q2)</f>
-        <v>129.80566066158457</v>
+        <v>130.67476534908457</v>
       </c>
       <c r="K24" s="34" t="s">
         <v>8</v>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="J25" s="48">
         <f>GammaG*MEdG+GammaQ*(Psi_0*MEd_Q1+MEd_Q2)</f>
-        <v>185.81615615777301</v>
+        <v>187.33708936089801</v>
       </c>
       <c r="K25" s="37" t="s">
         <v>18</v>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="J26" s="48">
         <f>GammaG*VEdG+GammaQ*(Psi_0*VEd_Q1+VEd_Q2)</f>
-        <v>106.18066066158457</v>
+        <v>107.04976534908457</v>
       </c>
       <c r="K26" s="40" t="s">
         <v>8</v>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="J30" s="54">
         <f>GammaG*qG+GammaQ*(qQ_1)</f>
-        <v>37.087331617595595</v>
+        <v>37.335647242595591</v>
       </c>
       <c r="K30" t="s">
         <v>7</v>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="J36" s="52">
         <f>MEd_U1/MplRd</f>
-        <v>0.68309500980417315</v>
+        <v>0.68766862448324662</v>
       </c>
       <c r="M36" s="41" t="s">
         <v>26</v>
@@ -2456,7 +2456,7 @@
       </c>
       <c r="J37" s="52">
         <f>VEd_U1/Q61</f>
-        <v>0.20043158842323336</v>
+        <v>0.20177356405152161</v>
       </c>
       <c r="M37" s="41" t="s">
         <v>92</v>
@@ -2470,7 +2470,7 @@
         <v>345</v>
       </c>
       <c r="P37" s="59">
-        <f t="shared" ref="P37:P41" si="4">N37*O37/1000</f>
+        <f t="shared" ref="P37:P40" si="4">N37*O37/1000</f>
         <v>0</v>
       </c>
       <c r="Q37" s="59">
@@ -2513,7 +2513,7 @@
         <v>2074.4468698294495</v>
       </c>
       <c r="S38" s="59">
-        <f t="shared" ref="S38:S41" si="6">S37+P38</f>
+        <f t="shared" ref="S38:S40" si="6">S37+P38</f>
         <v>1835.7449999999999</v>
       </c>
     </row>
@@ -2586,7 +2586,7 @@
         <v>101</v>
       </c>
       <c r="D41" s="6">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="E41" t="s">
         <v>2</v>
@@ -2598,7 +2598,7 @@
       </c>
       <c r="D42" s="77">
         <f>td</f>
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="E42" t="s">
         <v>2</v>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D49" s="47">
         <f>td*(d_1+d_2)/2000</f>
-        <v>0.40500000000000003</v>
+        <v>0.41249999999999998</v>
       </c>
       <c r="E49" t="s">
         <v>66</v>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="D50" s="9">
         <f>Ac*rhoC</f>
-        <v>1012.5000000000001</v>
+        <v>1031.25</v>
       </c>
       <c r="E50" t="s">
         <v>63</v>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="D51" s="9">
         <f>D50*9.81/1000</f>
-        <v>9.9326250000000016</v>
+        <v>10.116562500000001</v>
       </c>
       <c r="E51" t="s">
         <v>7</v>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="D55" s="81">
         <f>SUM(D51,D53)</f>
-        <v>10.805430827848586</v>
+        <v>10.989368327848585</v>
       </c>
       <c r="E55" s="57" t="s">
         <v>7</v>
@@ -3053,7 +3053,7 @@
       </c>
       <c r="N70" s="54">
         <f>5/384*qG*LL^4/(E*IncertieCM/100)*1000^2</f>
-        <v>13.72745657857409</v>
+        <v>13.961134817290295</v>
       </c>
       <c r="O70" t="s">
         <v>2</v>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="N74" s="54">
         <f>N70+N71+Psi_0*N72</f>
-        <v>32.783785933616507</v>
+        <v>33.017464172332716</v>
       </c>
       <c r="O74" t="s">
         <v>2</v>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="N79" s="56">
         <f>qG*LL/g*1000</f>
-        <v>7710.2972268032718</v>
+        <v>7841.5472268032718</v>
       </c>
       <c r="O79" t="s">
         <v>65</v>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="N82" s="56">
         <f>N79+N81*N80</f>
-        <v>9850.9700096778906</v>
+        <v>9982.2200096778906</v>
       </c>
       <c r="O82" t="s">
         <v>65</v>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="N84" s="56">
         <f>N82/2</f>
-        <v>4925.4850048389453</v>
+        <v>4991.1100048389453</v>
       </c>
       <c r="O84" t="s">
         <v>65</v>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="N86" s="54">
         <f>1/2/PI()*SQRT(PI()^4*(E*IncertieCM/100)/N82/LL^3)</f>
-        <v>4.2391110428015395</v>
+        <v>4.2111501116899834</v>
       </c>
       <c r="O86" t="s">
         <v>78</v>
@@ -3254,11 +3254,11 @@
       </c>
       <c r="F7" s="78">
         <f t="shared" ref="F7:F12" si="1">MEd_U1*E7*1000</f>
-        <v>-435.21362949767848</v>
+        <v>-438.12757179828776</v>
       </c>
       <c r="G7" s="97">
         <f t="shared" ref="G7:G12" si="2">ABS(F7/(FyS/GammaM0))</f>
-        <v>1.2614887811526914</v>
+        <v>1.2699349907196746</v>
       </c>
       <c r="I7" s="75"/>
       <c r="J7" s="4"/>
@@ -3280,11 +3280,11 @@
       </c>
       <c r="F8" s="78">
         <f t="shared" si="1"/>
-        <v>-398.38194112861692</v>
+        <v>-401.04927944564838</v>
       </c>
       <c r="G8" s="97">
         <f t="shared" si="2"/>
-        <v>1.1547302641409185</v>
+        <v>1.1624616795526039</v>
       </c>
       <c r="K8">
         <v>-138.15</v>
@@ -3329,11 +3329,11 @@
       </c>
       <c r="F10" s="78">
         <f t="shared" si="1"/>
-        <v>109.50765638159993</v>
+        <v>110.24085720653555</v>
       </c>
       <c r="G10" s="97">
         <f t="shared" si="2"/>
-        <v>0.31741349675826064</v>
+        <v>0.31953871654068278</v>
       </c>
       <c r="K10">
         <f>InertieY_MM4</f>
@@ -3353,11 +3353,11 @@
       </c>
       <c r="F11" s="78">
         <f t="shared" si="1"/>
-        <v>146.33934475066147</v>
+        <v>147.31914955917486</v>
       </c>
       <c r="G11" s="97">
         <f t="shared" si="2"/>
-        <v>0.42417201377003322</v>
+        <v>0.42701202770775321</v>
       </c>
     </row>
     <row r="12" spans="3:11" x14ac:dyDescent="0.25">
@@ -3374,11 +3374,11 @@
       </c>
       <c r="F12" s="78">
         <f t="shared" si="1"/>
-        <v>185.10954303388411</v>
+        <v>186.34893098300569</v>
       </c>
       <c r="G12" s="97">
         <f t="shared" si="2"/>
-        <v>0.53654940009821483</v>
+        <v>0.5401418289362484</v>
       </c>
     </row>
     <row r="13" spans="3:11" x14ac:dyDescent="0.25">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="D21" s="80">
         <f>qELU*df*6/tf^2/2</f>
-        <v>36.214084197236694</v>
+        <v>36.456553055443067</v>
       </c>
       <c r="E21" t="s">
         <v>43</v>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="L21" s="80">
         <f>qELU/2</f>
-        <v>18.543665808797797</v>
+        <v>18.667823621297796</v>
       </c>
       <c r="M21" t="s">
         <v>7</v>
@@ -3494,7 +3494,7 @@
       </c>
       <c r="L23" s="80">
         <f>qEdFl*(dbt/1000)</f>
-        <v>1.2516974420938514</v>
+        <v>1.2600780944376013</v>
       </c>
       <c r="M23" t="s">
         <v>161</v>
@@ -3533,22 +3533,22 @@
       </c>
       <c r="D25" s="59">
         <f>F10</f>
-        <v>109.50765638159993</v>
+        <v>110.24085720653555</v>
       </c>
       <c r="E25" s="66">
         <f>+D21</f>
-        <v>36.214084197236694</v>
+        <v>36.456553055443067</v>
       </c>
       <c r="F25" s="4">
         <v>0</v>
       </c>
       <c r="G25" s="78">
         <f>SQRT(D25^2+E25^2-D25*E25+3*F25^2)</f>
-        <v>96.63160565772354</v>
+        <v>97.278595789045553</v>
       </c>
       <c r="H25" s="98">
         <f t="shared" ref="H25:H30" si="3">G25/(FyS/GammaM0)</f>
-        <v>0.2800916106020972</v>
+        <v>0.28196694431607405</v>
       </c>
       <c r="K25" s="3"/>
     </row>
@@ -3558,29 +3558,29 @@
       </c>
       <c r="D26" s="59">
         <f>AVERAGE(D25,D27)</f>
-        <v>127.9235005661307</v>
+        <v>128.7800033828552</v>
       </c>
       <c r="E26" s="4">
         <v>0</v>
       </c>
       <c r="F26" s="75">
         <f>3/2*qELU/tf/2</f>
-        <v>1.4639736164840367</v>
+        <v>1.4737755490498259</v>
       </c>
       <c r="G26" s="78">
         <f t="shared" ref="G26:G30" si="4">SQRT(D26^2+E26^2-D26*E26+3*F26^2)</f>
-        <v>127.94862896233833</v>
+        <v>128.8053000244754</v>
       </c>
       <c r="H26" s="98">
         <f t="shared" si="3"/>
-        <v>0.37086559119518359</v>
+        <v>0.37334869572311713</v>
       </c>
       <c r="K26" s="3" t="s">
         <v>162</v>
       </c>
       <c r="L26" s="47">
         <f>(L23/L24)</f>
-        <v>5.0250810634463502E-2</v>
+        <v>5.0587261409032934E-2</v>
       </c>
     </row>
     <row r="27" spans="3:13" x14ac:dyDescent="0.25">
@@ -3589,22 +3589,22 @@
       </c>
       <c r="D27" s="59">
         <f>F11</f>
-        <v>146.33934475066147</v>
+        <v>147.31914955917486</v>
       </c>
       <c r="E27" s="66">
         <f>-E25</f>
-        <v>-36.214084197236694</v>
+        <v>-36.456553055443067</v>
       </c>
       <c r="F27" s="4">
         <v>0</v>
       </c>
       <c r="G27" s="78">
         <f t="shared" si="4"/>
-        <v>167.41030156016802</v>
+        <v>168.53118548063938</v>
       </c>
       <c r="H27" s="98">
         <f t="shared" si="3"/>
-        <v>0.48524725089903775</v>
+        <v>0.48849618979895471</v>
       </c>
       <c r="K27" s="3"/>
     </row>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="D28" s="59">
         <f>F11</f>
-        <v>146.33934475066147</v>
+        <v>147.31914955917486</v>
       </c>
       <c r="E28" s="66" t="e">
         <f>#REF!</f>
@@ -3639,22 +3639,22 @@
       </c>
       <c r="D29" s="59">
         <f>AVERAGE(D28,D30)</f>
-        <v>165.7244438922728</v>
+        <v>166.83404027109026</v>
       </c>
       <c r="E29" s="4">
         <v>0</v>
       </c>
       <c r="F29" s="66">
         <f>3/2*qELU/Pl_t/2</f>
-        <v>1.3907749356598349</v>
+        <v>1.4000867715973346</v>
       </c>
       <c r="G29" s="78">
         <f t="shared" si="4"/>
-        <v>165.74195023640831</v>
+        <v>166.85166382772385</v>
       </c>
       <c r="H29" s="98">
         <f t="shared" si="3"/>
-        <v>0.48041144996060381</v>
+        <v>0.48362801109485176</v>
       </c>
       <c r="K29" s="3"/>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="D30" s="59">
         <f>F12</f>
-        <v>185.10954303388411</v>
+        <v>186.34893098300569</v>
       </c>
       <c r="E30" s="66" t="e">
         <f>-E28</f>

</xml_diff>